<commit_message>
consultas adicionada: deputados, votacoes e proposicoes e alteração na função de chamda da API para adicionar o parametro de data
</commit_message>
<xml_diff>
--- a/partidos.xlsx
+++ b/partidos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,21 +512,21 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>38011</v>
+        <v>37901</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MISSÃO</t>
+          <t>NOVO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Partido Missão</t>
+          <t>Partido Novo</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/38011</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37901</t>
         </is>
       </c>
     </row>
@@ -535,21 +535,21 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>37901</v>
+        <v>36779</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>PCdoB</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Partido Novo</t>
+          <t>Partido Comunista do Brasil</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37901</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36779</t>
         </is>
       </c>
     </row>
@@ -558,21 +558,21 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>36779</v>
+        <v>36786</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PCdoB</t>
+          <t>PDT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Partido Comunista do Brasil</t>
+          <t>Partido Democrático Trabalhista</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36779</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36786</t>
         </is>
       </c>
     </row>
@@ -581,21 +581,21 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>36786</v>
+        <v>37906</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PDT</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Partido Democrático Trabalhista</t>
+          <t>Partido Liberal</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36786</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37906</t>
         </is>
       </c>
     </row>
@@ -604,21 +604,21 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>37906</v>
+        <v>36896</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PODE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Partido Liberal</t>
+          <t>Podemos</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37906</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36896</t>
         </is>
       </c>
     </row>
@@ -627,21 +627,21 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>36896</v>
+        <v>37903</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PODE</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Podemos</t>
+          <t>Progressistas</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36896</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37903</t>
         </is>
       </c>
     </row>
@@ -650,21 +650,21 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>37903</v>
+        <v>38010</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>PRD</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Progressistas</t>
+          <t>Partido Renovação Democrática</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37903</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/38010</t>
         </is>
       </c>
     </row>
@@ -673,21 +673,21 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>38010</v>
+        <v>36832</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PRD</t>
+          <t>PSB</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Partido Renovação Democrática</t>
+          <t>Partido Socialista Brasileiro</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/38010</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36832</t>
         </is>
       </c>
     </row>
@@ -696,21 +696,21 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>36832</v>
+        <v>36834</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PSB</t>
+          <t>PSD</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Partido Socialista Brasileiro</t>
+          <t>Partido Social Democrático</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36832</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36834</t>
         </is>
       </c>
     </row>
@@ -719,21 +719,21 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>36834</v>
+        <v>36835</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PSD</t>
+          <t>PSDB</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Partido Social Democrático</t>
+          <t>Partido da Social Democracia Brasileira</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36834</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36835</t>
         </is>
       </c>
     </row>
@@ -742,21 +742,21 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>36835</v>
+        <v>36839</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PSDB</t>
+          <t>PSOL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Partido da Social Democracia Brasileira</t>
+          <t>Partido Socialismo e Liberdade</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36835</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36839</t>
         </is>
       </c>
     </row>
@@ -765,21 +765,21 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>36839</v>
+        <v>36844</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PSOL</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Partido Socialismo e Liberdade</t>
+          <t>Partido dos Trabalhadores</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36839</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36844</t>
         </is>
       </c>
     </row>
@@ -788,21 +788,21 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>36844</v>
+        <v>36851</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Partido dos Trabalhadores</t>
+          <t>Partido Verde</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36844</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36851</t>
         </is>
       </c>
     </row>
@@ -811,21 +811,21 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>36851</v>
+        <v>36886</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>REDE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Partido Verde</t>
+          <t>Rede Sustentabilidade</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36851</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36886</t>
         </is>
       </c>
     </row>
@@ -834,21 +834,21 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>36886</v>
+        <v>37908</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>REDE</t>
+          <t>REPUBLICANOS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Rede Sustentabilidade</t>
+          <t>Republicanos</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/36886</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37908</t>
         </is>
       </c>
     </row>
@@ -857,21 +857,21 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>37908</v>
+        <v>37904</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>REPUBLICANOS</t>
+          <t>SOLIDARIEDADE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Republicanos</t>
+          <t>Solidariedade</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37908</t>
+          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37904</t>
         </is>
       </c>
     </row>
@@ -880,42 +880,19 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>37904</v>
+        <v>38009</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SOLIDARIEDADE</t>
+          <t>UNIÃO</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Solidariedade</t>
+          <t>União Brasil</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
-        <is>
-          <t>https://dadosabertos.camara.leg.br/api/v2/partidos/37904</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" t="n">
-        <v>38009</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>UNIÃO</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>União Brasil</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
         <is>
           <t>https://dadosabertos.camara.leg.br/api/v2/partidos/38009</t>
         </is>

</xml_diff>